<commit_message>
Sync planning SharePoint : S37
</commit_message>
<xml_diff>
--- a/Plannings 2026 S37.xlsx
+++ b/Plannings 2026 S37.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F595FD38-6611-4D01-B273-82F362A96CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{F595FD38-6611-4D01-B273-82F362A96CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5259B5EB-BC75-4817-9100-C8B3560796CC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -244,9 +244,6 @@
     <t>19:00/00:30+</t>
   </si>
   <si>
-    <t>15:45/16:45</t>
-  </si>
-  <si>
     <t>FREIXEDAS-BERENGUER Maxime</t>
   </si>
   <si>
@@ -392,6 +389,9 @@
   </si>
   <si>
     <t>EDF // ANNIV</t>
+  </si>
+  <si>
+    <t>15:45/17:30</t>
   </si>
 </sst>
 </file>
@@ -4706,25 +4706,25 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="E3" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="G3" s="15" t="s">
-        <v>118</v>
-      </c>
       <c r="H3" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5381,7 +5381,7 @@
         <v>45</v>
       </c>
       <c r="E45" s="39" t="s">
-        <v>69</v>
+        <v>118</v>
       </c>
       <c r="F45" s="46"/>
       <c r="G45" s="1"/>
@@ -5413,7 +5413,7 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="20" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B48" s="21"/>
       <c r="C48" s="21"/>
@@ -5467,7 +5467,7 @@
     </row>
     <row r="52" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B52" s="26"/>
       <c r="C52" s="27"/>
@@ -5479,7 +5479,7 @@
     </row>
     <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B53" s="26"/>
       <c r="C53" s="27"/>
@@ -5491,7 +5491,7 @@
     </row>
     <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B54" s="26"/>
       <c r="C54" s="27"/>
@@ -5503,7 +5503,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B55" s="21"/>
       <c r="C55" s="21"/>
@@ -5529,7 +5529,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B57" s="21" t="s">
         <v>19</v>
@@ -5546,7 +5546,7 @@
     <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="23"/>
       <c r="B58" s="24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C58" s="24"/>
       <c r="D58" s="24" t="s">
@@ -5559,7 +5559,7 @@
     </row>
     <row r="59" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B59" s="26"/>
       <c r="C59" s="27"/>
@@ -5571,7 +5571,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B60" s="21"/>
       <c r="C60" s="21"/>
@@ -5579,7 +5579,7 @@
       <c r="E60" s="21"/>
       <c r="F60" s="21"/>
       <c r="G60" s="52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H60" s="22" t="s">
         <v>19</v>
@@ -5593,10 +5593,10 @@
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="53" t="s">
+        <v>79</v>
+      </c>
+      <c r="H61" s="30" t="s">
         <v>80</v>
-      </c>
-      <c r="H61" s="30" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -5610,7 +5610,7 @@
         <v>19</v>
       </c>
       <c r="H62" s="50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -5621,7 +5621,7 @@
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H63" s="49" t="s">
         <v>47</v>
@@ -5648,7 +5648,7 @@
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
       <c r="H65" s="30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -5660,7 +5660,7 @@
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
       <c r="H66" s="50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5677,7 +5677,7 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B68" s="21"/>
       <c r="C68" s="21"/>
@@ -5703,7 +5703,7 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B70" s="21" t="s">
         <v>19</v>
@@ -5719,27 +5719,27 @@
         <v>19</v>
       </c>
       <c r="G70" s="42" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H70" s="22"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="29"/>
       <c r="B71" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="D71" s="1"/>
       <c r="E71" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F71" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G71" s="41" t="s">
         <v>89</v>
-      </c>
-      <c r="G71" s="41" t="s">
-        <v>90</v>
       </c>
       <c r="H71" s="30"/>
     </row>
@@ -5767,13 +5767,13 @@
         <v>24</v>
       </c>
       <c r="G73" s="24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H73" s="25"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B74" s="21"/>
       <c r="C74" s="21"/>
@@ -5782,7 +5782,7 @@
       <c r="F74" s="21"/>
       <c r="G74" s="21"/>
       <c r="H74" s="48" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -5794,7 +5794,7 @@
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
       <c r="H75" s="49" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -5818,12 +5818,12 @@
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B78" s="26"/>
       <c r="C78" s="27"/>
@@ -5835,7 +5835,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B79" s="21"/>
       <c r="C79" s="21" t="s">
@@ -5853,7 +5853,7 @@
       <c r="A80" s="23"/>
       <c r="B80" s="24"/>
       <c r="C80" s="24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D80" s="24"/>
       <c r="E80" s="24"/>
@@ -5865,7 +5865,7 @@
     </row>
     <row r="81" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B81" s="26"/>
       <c r="C81" s="27"/>
@@ -5934,7 +5934,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -5942,7 +5942,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -5953,16 +5953,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>103</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -6171,7 +6171,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B19" s="7">
         <v>0</v>
@@ -6188,7 +6188,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B20" s="7">
         <v>0</v>
@@ -6205,7 +6205,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B21" s="7">
         <v>0</v>
@@ -6222,7 +6222,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B22" s="7">
         <v>0</v>
@@ -6239,7 +6239,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B23" s="7">
         <v>0</v>
@@ -6256,7 +6256,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B24" s="7">
         <v>0</v>
@@ -6273,7 +6273,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" s="7">
         <v>0</v>
@@ -6290,7 +6290,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B26" s="7">
         <v>0</v>
@@ -6307,7 +6307,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B27" s="7">
         <v>0</v>
@@ -6324,7 +6324,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B28" s="7">
         <v>0</v>
@@ -6341,7 +6341,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B29" s="7">
         <v>0</v>
@@ -6358,7 +6358,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B30" s="7">
         <v>0</v>
@@ -6375,7 +6375,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B31" s="7">
         <v>0</v>
@@ -6392,7 +6392,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B32" s="7">
         <v>0</v>
@@ -6442,40 +6442,40 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>105</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>109</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>111</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -6656,13 +6656,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8B9DAAF-0AE9-45EC-8679-4102E750C10E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{277BEA7E-E313-484E-A6A5-7996405961DB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA508A95-29A9-4047-9E07-846F082FDF78}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{030C3010-3A1B-4E5B-AD5F-3D421DE782BD}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6E0040D-1B66-4370-9E48-5C2583DE331D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{287291FB-E397-446F-982C-CD5E80DC76D3}"/>
 </file>
</xml_diff>